<commit_message>
Move BAro box deneme
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -310,6 +310,43 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BAro box deneme</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>9</v>
+      </c>
+      <c r="H2">
+        <v>81</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Delete BAro box deneme
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -310,43 +310,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BAro box deneme</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grid</t>
-        </is>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>9</v>
-      </c>
-      <c r="H2">
-        <v>81</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>81</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move UMUT CAA CELLS
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -313,17 +313,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
+          <t xml:space="preserve">UMUT CAA CELLS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -360,7 +360,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CAA CELLS</t>
+          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
Move UMUT CELLS -80
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -350,17 +350,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
+          <t xml:space="preserve">UMUT CELLS -80</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -397,7 +397,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -80</t>
+          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>

<commit_message>
Move UMUT CELLS -4-
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -461,17 +461,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Freezer 1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not placed yet</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -508,7 +508,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">

</xml_diff>

<commit_message>
Delete Baro CELLS #1 (-80)
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -532,43 +532,6 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not placed yet</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not placed yet</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Baro CELLS #1 (-80)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grid</t>
-        </is>
-      </c>
-      <c r="F8">
-        <v>9</v>
-      </c>
-      <c r="G8">
-        <v>9</v>
-      </c>
-      <c r="H8">
-        <v>81</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>81</v>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Import 506 vials from CAA Lab-Cell Stocks (-80 & LiqNitro)-2 NEW.xlsx from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -828,6 +828,117 @@
         <v>81</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beyza Caa Hücre Box 1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F16">
+        <v>9</v>
+      </c>
+      <c r="G16">
+        <v>9</v>
+      </c>
+      <c r="H16">
+        <v>81</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beyza Caa Sıvı Azot Box 1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F17">
+        <v>9</v>
+      </c>
+      <c r="G17">
+        <v>9</v>
+      </c>
+      <c r="H17">
+        <v>81</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not placed yet</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Beyza Caa Hücre Box 2</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid</t>
+        </is>
+      </c>
+      <c r="F18">
+        <v>9</v>
+      </c>
+      <c r="G18">
+        <v>9</v>
+      </c>
+      <c r="H18">
+        <v>81</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Delete a koox rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -199,11 +199,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -281,11 +276,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -363,11 +353,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -445,11 +430,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -527,11 +507,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -609,11 +584,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -691,11 +661,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M8" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -773,11 +738,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -855,11 +815,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -937,11 +892,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1019,11 +969,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M12" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1101,11 +1046,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1183,11 +1123,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1265,11 +1200,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1347,11 +1277,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1429,11 +1354,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1511,11 +1431,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1593,11 +1508,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1675,11 +1585,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1757,11 +1662,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1839,11 +1739,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1921,11 +1816,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2003,11 +1893,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2085,11 +1970,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2167,11 +2047,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2249,11 +2124,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2331,11 +2201,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M28" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2413,11 +2278,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2495,11 +2355,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2577,11 +2432,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M31" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2659,11 +2509,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M32" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2751,11 +2596,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2843,11 +2683,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M34" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2935,11 +2770,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3027,11 +2857,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3109,11 +2934,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M37" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3601,11 +3421,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M43" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4011,11 +3826,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M48" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4175,11 +3985,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M50" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4257,11 +4062,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M51" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4339,11 +4139,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M52" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4421,11 +4216,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M53" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4503,11 +4293,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M54" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4585,11 +4370,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M55" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4667,11 +4447,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M56" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4749,11 +4524,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M57" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4831,11 +4601,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M58" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4913,11 +4678,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M59" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5005,11 +4765,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M60" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5097,11 +4852,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5189,11 +4939,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M62" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5281,11 +5026,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M63" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5363,11 +5103,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M64" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5445,11 +5180,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M65" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5527,11 +5257,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5609,11 +5334,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5691,11 +5411,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5773,11 +5488,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5865,11 +5575,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5947,11 +5652,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6029,11 +5729,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6111,11 +5806,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6521,11 +6211,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M78" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6603,11 +6288,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M79" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6685,11 +6365,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M80" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6767,11 +6442,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M81" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6849,11 +6519,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M82" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6931,11 +6596,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M83" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7013,11 +6673,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M84" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7095,11 +6750,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M85" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7177,11 +6827,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M86" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7341,11 +6986,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M88" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7433,11 +7073,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M89" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8171,11 +7806,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M98" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8499,11 +8129,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M102" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8581,11 +8206,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M103" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8663,11 +8283,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M104" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9165,11 +8780,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M110" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9329,11 +8939,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M112" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9411,11 +9016,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M113" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9493,11 +9093,6 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M114" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9575,11 +9170,6 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
-      <c r="L115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M115" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9657,11 +9247,6 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M116" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9739,11 +9324,6 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
-      <c r="L117" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M117" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9821,11 +9401,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M118" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -9903,11 +9478,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M119" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10149,11 +9719,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M122" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10231,11 +9796,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M123" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10313,11 +9873,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M124" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10395,11 +9950,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M125" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -10477,11 +10027,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M126" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -10559,11 +10104,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M127" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10641,11 +10181,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M128" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10723,11 +10258,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M129" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10805,11 +10335,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M130" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10887,11 +10412,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M131" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10969,11 +10489,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M132" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11051,11 +10566,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M133" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11133,11 +10643,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M134" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11215,11 +10720,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M135" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11297,11 +10797,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M136" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11379,11 +10874,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M137" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11461,11 +10951,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M138" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11543,11 +11028,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M139" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11625,11 +11105,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M140" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11707,11 +11182,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M141" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11789,11 +11259,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M142" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11871,11 +11336,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M143" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11953,11 +11413,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M144" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -12035,11 +11490,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M145" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12117,11 +11567,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M146" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12199,11 +11644,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M147" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12281,11 +11721,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M148" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12363,11 +11798,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M149" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12445,11 +11875,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M150" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12527,11 +11952,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M151" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12609,11 +12029,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M152" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12691,11 +12106,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M153" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -13946,11 +13356,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L168" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M168" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -14192,11 +13597,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M171" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -14274,11 +13674,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L172" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M172" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14602,11 +13997,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M176" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14684,11 +14074,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M177" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14766,11 +14151,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M178" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14848,11 +14228,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M179" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15012,11 +14387,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M181" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15094,11 +14464,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M182" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15186,11 +14551,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L183" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M183" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15268,11 +14628,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M184" t="inlineStr">
         <is>
           <t xml:space="preserve">EnzaR</t>
@@ -15350,11 +14705,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L185" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M185" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15442,11 +14792,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M186" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15534,11 +14879,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L187" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M187" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15626,11 +14966,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L188" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M188" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15708,11 +15043,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M189" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16200,11 +15530,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L195" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M195" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -16364,11 +15689,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L197" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M197" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -16446,11 +15766,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L198" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M198" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -16528,11 +15843,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L199" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M199" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16610,11 +15920,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L200" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M200" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16692,11 +15997,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L201" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M201" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16774,11 +16074,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M202" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16856,11 +16151,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L203" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M203" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16938,11 +16228,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L204" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M204" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -17020,11 +16305,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L205" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M205" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -17102,11 +16382,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L206" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M206" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -17184,11 +16459,6 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L207" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M207" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -17266,11 +16536,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L208" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M208" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17348,11 +16613,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L209" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M209" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17430,11 +16690,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L210" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M210" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17512,11 +16767,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L211" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M211" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17594,11 +16844,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L212" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M212" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17686,11 +16931,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L213" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M213" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17768,11 +17008,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L214" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M214" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17850,11 +17085,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M215" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17942,11 +17172,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M216" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19346,11 +18571,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L233" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M233" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19428,11 +18648,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L234" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M234" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19674,11 +18889,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L237" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M237" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19997,11 +19207,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L241" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M241" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20074,11 +19279,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L242" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M242" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20156,11 +19356,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M243" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20238,11 +19433,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L244" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M244" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20320,11 +19510,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L245" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M245" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20402,11 +19587,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L246" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M246" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20479,11 +19659,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L247" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M247" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20561,11 +19736,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L248" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M248" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20643,11 +19813,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L249" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M249" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20725,11 +19890,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M250" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20807,11 +19967,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L251" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M251" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20889,11 +20044,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M252" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20971,11 +20121,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L253" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M253" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21053,11 +20198,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M254" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21135,11 +20275,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M255" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21217,11 +20352,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L256" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M256" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21299,11 +20429,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M257" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21381,11 +20506,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M258" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21463,11 +20583,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L259" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M259" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21709,11 +20824,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M262" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21791,11 +20901,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M263" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21873,11 +20978,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M264" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21955,11 +21055,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M265" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22037,11 +21132,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M266" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22119,11 +21209,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M267" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22196,11 +21281,6 @@
           <t xml:space="preserve">22-06-26</t>
         </is>
       </c>
-      <c r="L268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M268" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -22273,11 +21353,6 @@
           <t xml:space="preserve">22-06-26</t>
         </is>
       </c>
-      <c r="L269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M269" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -22355,11 +21430,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M270" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -22427,11 +21497,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="L271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M271" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -22509,11 +21574,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L272" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M272" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22591,11 +21651,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L273" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M273" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22673,11 +21728,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M274" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22755,11 +21805,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M275" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22837,11 +21882,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M276" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22919,11 +21959,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M277" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23001,11 +22036,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M278" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23083,11 +22113,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M279" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23165,11 +22190,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M280" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23980,11 +23000,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M290" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24062,11 +23077,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M291" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24144,11 +23154,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M292" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24308,11 +23313,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M294" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24718,11 +23718,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L299" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M299" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24800,11 +23795,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L300" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M300" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24882,11 +23872,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M301" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24964,11 +23949,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L302" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M302" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25046,11 +24026,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L303" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M303" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25128,11 +24103,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L304" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M304" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -25210,11 +24180,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L305" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M305" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -25292,11 +24257,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L306" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M306" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -25374,11 +24334,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L307" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M307" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -26358,11 +25313,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L319" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M319" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26440,11 +25390,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L320" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M320" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26850,11 +25795,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L325" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M325" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26932,11 +25872,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L326" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M326" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27024,11 +25959,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M327" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27116,11 +26046,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L328" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M328" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27198,11 +26123,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L329" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M329" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27280,11 +26200,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L330" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M330" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27362,11 +26277,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L331" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M331" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27444,11 +26354,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L332" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M332" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27521,11 +26426,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L333" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M333" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27603,11 +26503,6 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
-      <c r="L334" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M334" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27931,11 +26826,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L338" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M338" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28013,11 +26903,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M339" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28095,11 +26980,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L340" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M340" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28423,11 +27303,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L344" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M344" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28505,11 +27380,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L345" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M345" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28587,11 +27457,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L346" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M346" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28669,11 +27534,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L347" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M347" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28751,11 +27611,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L348" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M348" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28833,11 +27688,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L349" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M349" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -28915,11 +27765,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L350" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M350" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28997,11 +27842,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L351" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M351" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -29079,11 +27919,6 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
-      <c r="L352" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M352" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -29141,11 +27976,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L353" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M353" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29389,11 +28219,6 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L357" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M357" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29637,11 +28462,6 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
-      <c r="L361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M361" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29741,11 +28561,6 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L363" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M363" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29793,11 +28608,6 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M364" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29845,11 +28655,6 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M365" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29897,11 +28702,6 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="L366" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M366" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -29949,11 +28749,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="L367" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M367" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -30001,11 +28796,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="L368" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
       <c r="M368" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -30051,11 +28841,6 @@
       <c r="I369" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-09</t>
-        </is>
-      </c>
-      <c r="L369" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">

</xml_diff>

<commit_message>
Add a koox catch-all rule: no KO/OX/CASPEX/FLAG in the name reads as WT
A name with no koox marker in it (Du145, Huh7, LnCap, ...) had no rule
that could ever cover it -- classification only reads the name's text,
and there was nothing there to match -- so these sat in Review's
"Names no rule covers" list permanently, no matter what rule got
added. DEFAULT_RULES already carries exactly this catch-all
({ value: "WT" }, sorted last) but the lab's own lab-rules.json never
had it.

Restores it. 1526 vials across the lab now read koox=WT instead of
unmatched; none of them are affected if a facet was ever pinned by
hand. Every member's cellstocks/data/*.xlsx is regenerated in this
same commit so CI's "workbook still matches its inventory" check
stays true.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W7agPBsFxuZZB7B72D8K1E
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -199,6 +199,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -276,6 +281,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -353,6 +363,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -430,6 +445,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -507,6 +527,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -584,6 +609,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -661,6 +691,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -738,6 +773,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -815,6 +855,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -892,6 +937,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -969,6 +1019,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1046,6 +1101,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1123,6 +1183,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1200,6 +1265,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1277,6 +1347,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1354,6 +1429,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1431,6 +1511,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1508,6 +1593,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1585,6 +1675,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1662,6 +1757,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M21" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1739,6 +1839,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M22" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1816,6 +1921,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1893,6 +2003,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -1970,6 +2085,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2047,6 +2167,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M26" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2124,6 +2249,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2201,6 +2331,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2278,6 +2413,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M29" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2355,6 +2495,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M30" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2432,6 +2577,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M31" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2509,6 +2659,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2596,6 +2751,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M33" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2683,6 +2843,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M34" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2770,6 +2935,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M35" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2857,6 +3027,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -2934,6 +3109,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M37" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3421,6 +3601,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M43" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3826,6 +4011,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M48" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -3985,6 +4175,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M50" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4062,6 +4257,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M51" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4139,6 +4339,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M52" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4216,6 +4421,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M53" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4293,6 +4503,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M54" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4370,6 +4585,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4447,6 +4667,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M56" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4524,6 +4749,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M57" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4601,6 +4831,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M58" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4678,6 +4913,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M59" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4765,6 +5005,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M60" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4852,6 +5097,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -4939,6 +5189,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M62" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5026,6 +5281,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M63" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5103,6 +5363,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M64" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5180,6 +5445,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M65" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5257,6 +5527,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5334,6 +5609,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5411,6 +5691,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M68" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5488,6 +5773,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M69" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -5575,6 +5865,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M70" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5652,6 +5947,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M71" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5729,6 +6029,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M72" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -5806,6 +6111,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M73" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6211,6 +6521,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M78" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6288,6 +6603,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M79" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6365,6 +6685,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M80" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6442,6 +6767,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M81" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6519,6 +6849,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M82" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6596,6 +6931,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M83" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6673,6 +7013,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M84" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6750,6 +7095,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M85" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6827,6 +7177,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M86" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -6986,6 +7341,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M88" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7073,6 +7433,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M89" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -7806,6 +8171,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M98" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8129,6 +8499,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M102" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8206,6 +8581,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M103" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8283,6 +8663,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M104" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8780,6 +9165,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M110" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -8939,6 +9329,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M112" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9016,6 +9411,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M113" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9093,6 +9493,11 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M114" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9170,6 +9575,11 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M115" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9247,6 +9657,11 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M116" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9324,6 +9739,11 @@
           <t xml:space="preserve">HepG2</t>
         </is>
       </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M117" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9401,6 +9821,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M118" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -9478,6 +9903,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M119" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9719,6 +10149,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M122" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9796,6 +10231,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M123" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9873,6 +10313,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M124" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -9950,6 +10395,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M125" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -10027,6 +10477,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M126" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -10104,6 +10559,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M127" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10181,6 +10641,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M128" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10258,6 +10723,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M129" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10335,6 +10805,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M130" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10412,6 +10887,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M131" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10489,6 +10969,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M132" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10566,6 +11051,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M133" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10643,6 +11133,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M134" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10720,6 +11215,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M135" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10797,6 +11297,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M136" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -10874,6 +11379,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M137" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -10951,6 +11461,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M138" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11028,6 +11543,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M139" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11105,6 +11625,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M140" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11182,6 +11707,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M141" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11259,6 +11789,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M142" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11336,6 +11871,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M143" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11413,6 +11953,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M144" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -11490,6 +12035,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M145" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11567,6 +12117,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M146" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11644,6 +12199,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M147" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11721,6 +12281,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M148" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11798,6 +12363,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M149" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11875,6 +12445,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M150" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -11952,6 +12527,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M151" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12029,6 +12609,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M152" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -12106,6 +12691,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M153" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -13356,6 +13946,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M168" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -13597,6 +14192,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M171" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -13674,6 +14274,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M172" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -13997,6 +14602,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M176" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14074,6 +14684,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M177" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14151,6 +14766,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M178" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14228,6 +14848,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M179" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14387,6 +15012,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M181" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14464,6 +15094,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M182" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14551,6 +15186,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M183" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14628,6 +15268,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M184" t="inlineStr">
         <is>
           <t xml:space="preserve">EnzaR</t>
@@ -14705,6 +15350,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M185" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14792,6 +15442,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M186" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14879,6 +15534,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M187" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -14966,6 +15626,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M188" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15043,6 +15708,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M189" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -15530,6 +16200,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M195" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -15689,6 +16364,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M197" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -15766,6 +16446,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M198" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -15843,6 +16528,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M199" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -15920,6 +16610,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M200" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -15997,6 +16692,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M201" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16074,6 +16774,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M202" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16151,6 +16856,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M203" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16228,6 +16938,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M204" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16305,6 +17020,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M205" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16382,6 +17102,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M206" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16459,6 +17184,11 @@
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M207" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
@@ -16536,6 +17266,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M208" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16613,6 +17348,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M209" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16690,6 +17430,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M210" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16767,6 +17512,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M211" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16844,6 +17594,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M212" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -16931,6 +17686,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M213" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17008,6 +17768,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M214" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17085,6 +17850,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M215" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -17172,6 +17942,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M216" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -18571,6 +19346,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M233" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -18648,6 +19428,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M234" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -18889,6 +19674,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M237" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19207,6 +19997,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M241" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19279,6 +20074,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M242" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19356,6 +20156,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M243" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19433,6 +20238,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M244" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19510,6 +20320,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M245" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19587,6 +20402,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M246" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19659,6 +20479,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M247" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19736,6 +20561,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M248" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19813,6 +20643,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M249" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19890,6 +20725,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M250" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -19967,6 +20807,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M251" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20044,6 +20889,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M252" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20121,6 +20971,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M253" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20198,6 +21053,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M254" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -20275,6 +21135,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M255" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20352,6 +21217,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M256" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20429,6 +21299,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M257" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -20506,6 +21381,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M258" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20583,6 +21463,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M259" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -20824,6 +21709,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M262" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -20901,6 +21791,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M263" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -20978,6 +21873,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M264" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21055,6 +21955,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M265" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21132,6 +22037,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M266" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21209,6 +22119,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M267" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21281,6 +22196,11 @@
           <t xml:space="preserve">22-06-26</t>
         </is>
       </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M268" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21353,6 +22273,11 @@
           <t xml:space="preserve">22-06-26</t>
         </is>
       </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M269" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21430,6 +22355,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M270" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21497,6 +22427,11 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M271" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -21574,6 +22509,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M272" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21651,6 +22591,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M273" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21728,6 +22673,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M274" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21805,6 +22755,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M275" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21882,6 +22837,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M276" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -21959,6 +22919,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M277" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22036,6 +23001,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M278" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22113,6 +23083,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M279" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -22190,6 +23165,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M280" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23000,6 +23980,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M290" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -23077,6 +24062,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M291" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -23154,6 +24144,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M292" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -23313,6 +24308,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M294" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -23718,6 +24718,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M299" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23795,6 +24800,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M300" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23872,6 +24882,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M301" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -23949,6 +24964,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M302" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24026,6 +25046,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M303" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -24103,6 +25128,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M304" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24180,6 +25210,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M305" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24257,6 +25292,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M306" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -24334,6 +25374,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M307" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -25313,6 +26358,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M319" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25390,6 +26440,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M320" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25795,6 +26850,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M325" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25872,6 +26932,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M326" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -25959,6 +27024,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M327" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26046,6 +27116,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M328" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26123,6 +27198,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M329" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26200,6 +27280,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M330" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26277,6 +27362,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M331" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26354,6 +27444,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M332" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26426,6 +27521,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M333" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26503,6 +27603,11 @@
           <t xml:space="preserve">LnCap</t>
         </is>
       </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M334" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26826,6 +27931,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M338" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26903,6 +28013,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M339" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -26980,6 +28095,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M340" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27303,6 +28423,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M344" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27380,6 +28505,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M345" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27457,6 +28587,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M346" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27534,6 +28669,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M347" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27611,6 +28751,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M348" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27688,6 +28833,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M349" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27765,6 +28915,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M350" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -27842,6 +28997,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M351" t="inlineStr">
         <is>
           <t xml:space="preserve">CisR</t>
@@ -27919,6 +29079,11 @@
           <t xml:space="preserve">Du145</t>
         </is>
       </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M352" t="inlineStr">
         <is>
           <t xml:space="preserve">DtxR</t>
@@ -27976,6 +29141,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M353" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28219,6 +29389,11 @@
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M357" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28462,6 +29637,11 @@
           <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M361" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28561,6 +29741,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M363" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28608,6 +29793,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M364" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28655,6 +29845,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M365" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28702,6 +29897,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M366" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28749,6 +29949,11 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M367" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28796,6 +30001,11 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
       <c r="M368" t="inlineStr">
         <is>
           <t xml:space="preserve">-</t>
@@ -28841,6 +30051,11 @@
       <c r="I369" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">

</xml_diff>

<commit_message>
Add a origin rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -30053,6 +30053,11 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
       <c r="L369" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>

</xml_diff>

<commit_message>
Edit a koox rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -201,7 +201,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -283,7 +283,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -365,7 +365,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -4177,7 +4177,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -4423,7 +4423,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4751,7 +4751,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -5099,7 +5099,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -5191,7 +5191,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -5365,7 +5365,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5529,7 +5529,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5611,7 +5611,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5867,7 +5867,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -6031,7 +6031,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -6523,7 +6523,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -6687,7 +6687,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6769,7 +6769,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -6851,7 +6851,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -7015,7 +7015,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -7179,7 +7179,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -7343,7 +7343,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -8501,7 +8501,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -9331,7 +9331,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -9413,7 +9413,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
@@ -9495,7 +9495,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
@@ -9741,7 +9741,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M117" t="inlineStr">
@@ -9823,7 +9823,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -10151,7 +10151,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
@@ -10315,7 +10315,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
@@ -10479,7 +10479,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
@@ -10561,7 +10561,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
@@ -10807,7 +10807,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
@@ -11053,7 +11053,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M133" t="inlineStr">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
@@ -11217,7 +11217,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
@@ -11299,7 +11299,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
@@ -11545,7 +11545,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -11709,7 +11709,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -11791,7 +11791,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -11873,7 +11873,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
@@ -12037,7 +12037,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -12201,7 +12201,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
@@ -12365,7 +12365,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
@@ -12529,7 +12529,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
@@ -14194,7 +14194,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
@@ -14276,7 +14276,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M172" t="inlineStr">
@@ -14604,7 +14604,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
@@ -14686,7 +14686,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
@@ -14768,7 +14768,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M179" t="inlineStr">
@@ -15014,7 +15014,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
@@ -15352,7 +15352,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M186" t="inlineStr">
@@ -15536,7 +15536,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
@@ -15628,7 +15628,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
@@ -15710,7 +15710,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M189" t="inlineStr">
@@ -16202,7 +16202,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M195" t="inlineStr">
@@ -16366,7 +16366,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M197" t="inlineStr">
@@ -16448,7 +16448,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M198" t="inlineStr">
@@ -16530,7 +16530,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
@@ -16612,7 +16612,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -16694,7 +16694,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -16776,7 +16776,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -16858,7 +16858,7 @@
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
@@ -16940,7 +16940,7 @@
       </c>
       <c r="L204" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
@@ -17022,7 +17022,7 @@
       </c>
       <c r="L205" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
@@ -17186,7 +17186,7 @@
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
@@ -17350,7 +17350,7 @@
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
@@ -17596,7 +17596,7 @@
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M212" t="inlineStr">
@@ -17688,7 +17688,7 @@
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M213" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="L214" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M214" t="inlineStr">
@@ -17852,7 +17852,7 @@
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M215" t="inlineStr">
@@ -17944,7 +17944,7 @@
       </c>
       <c r="L216" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M216" t="inlineStr">
@@ -19348,7 +19348,7 @@
       </c>
       <c r="L233" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M233" t="inlineStr">
@@ -19430,7 +19430,7 @@
       </c>
       <c r="L234" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M234" t="inlineStr">
@@ -19676,7 +19676,7 @@
       </c>
       <c r="L237" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M237" t="inlineStr">
@@ -19999,7 +19999,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
@@ -20076,7 +20076,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
@@ -20158,7 +20158,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
@@ -20240,7 +20240,7 @@
       </c>
       <c r="L244" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M244" t="inlineStr">
@@ -20322,7 +20322,7 @@
       </c>
       <c r="L245" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M245" t="inlineStr">
@@ -20404,7 +20404,7 @@
       </c>
       <c r="L246" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M246" t="inlineStr">
@@ -20481,7 +20481,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M247" t="inlineStr">
@@ -20563,7 +20563,7 @@
       </c>
       <c r="L248" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M248" t="inlineStr">
@@ -20645,7 +20645,7 @@
       </c>
       <c r="L249" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M249" t="inlineStr">
@@ -20727,7 +20727,7 @@
       </c>
       <c r="L250" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M250" t="inlineStr">
@@ -20809,7 +20809,7 @@
       </c>
       <c r="L251" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M251" t="inlineStr">
@@ -20891,7 +20891,7 @@
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M252" t="inlineStr">
@@ -20973,7 +20973,7 @@
       </c>
       <c r="L253" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M253" t="inlineStr">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="L254" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M254" t="inlineStr">
@@ -21137,7 +21137,7 @@
       </c>
       <c r="L255" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M255" t="inlineStr">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="L256" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M256" t="inlineStr">
@@ -21301,7 +21301,7 @@
       </c>
       <c r="L257" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M257" t="inlineStr">
@@ -21383,7 +21383,7 @@
       </c>
       <c r="L258" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M258" t="inlineStr">
@@ -21465,7 +21465,7 @@
       </c>
       <c r="L259" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M259" t="inlineStr">
@@ -21711,7 +21711,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M262" t="inlineStr">
@@ -21793,7 +21793,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M263" t="inlineStr">
@@ -21875,7 +21875,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M264" t="inlineStr">
@@ -21957,7 +21957,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M265" t="inlineStr">
@@ -22039,7 +22039,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M266" t="inlineStr">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M267" t="inlineStr">
@@ -22198,7 +22198,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M268" t="inlineStr">
@@ -22275,7 +22275,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M269" t="inlineStr">
@@ -22357,7 +22357,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M270" t="inlineStr">
@@ -22429,7 +22429,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M271" t="inlineStr">
@@ -22511,7 +22511,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M272" t="inlineStr">
@@ -22593,7 +22593,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M273" t="inlineStr">
@@ -22675,7 +22675,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M274" t="inlineStr">
@@ -22757,7 +22757,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M275" t="inlineStr">
@@ -22839,7 +22839,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M276" t="inlineStr">
@@ -22921,7 +22921,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M277" t="inlineStr">
@@ -23003,7 +23003,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M278" t="inlineStr">
@@ -23085,7 +23085,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M279" t="inlineStr">
@@ -23167,7 +23167,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M280" t="inlineStr">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="L290" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M290" t="inlineStr">
@@ -24064,7 +24064,7 @@
       </c>
       <c r="L291" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M291" t="inlineStr">
@@ -24146,7 +24146,7 @@
       </c>
       <c r="L292" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M292" t="inlineStr">
@@ -24310,7 +24310,7 @@
       </c>
       <c r="L294" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M294" t="inlineStr">
@@ -24720,7 +24720,7 @@
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
@@ -24802,7 +24802,7 @@
       </c>
       <c r="L300" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M300" t="inlineStr">
@@ -24884,7 +24884,7 @@
       </c>
       <c r="L301" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M301" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M302" t="inlineStr">
@@ -25048,7 +25048,7 @@
       </c>
       <c r="L303" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M303" t="inlineStr">
@@ -25130,7 +25130,7 @@
       </c>
       <c r="L304" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M304" t="inlineStr">
@@ -25212,7 +25212,7 @@
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M305" t="inlineStr">
@@ -25294,7 +25294,7 @@
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M306" t="inlineStr">
@@ -25376,7 +25376,7 @@
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
@@ -26360,7 +26360,7 @@
       </c>
       <c r="L319" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M319" t="inlineStr">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
@@ -26852,7 +26852,7 @@
       </c>
       <c r="L325" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M325" t="inlineStr">
@@ -26934,7 +26934,7 @@
       </c>
       <c r="L326" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M326" t="inlineStr">
@@ -27026,7 +27026,7 @@
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M327" t="inlineStr">
@@ -27118,7 +27118,7 @@
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M328" t="inlineStr">
@@ -27200,7 +27200,7 @@
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M329" t="inlineStr">
@@ -27282,7 +27282,7 @@
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
@@ -27364,7 +27364,7 @@
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
@@ -27446,7 +27446,7 @@
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
@@ -27523,7 +27523,7 @@
       </c>
       <c r="L333" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M333" t="inlineStr">
@@ -27605,7 +27605,7 @@
       </c>
       <c r="L334" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M334" t="inlineStr">
@@ -27933,7 +27933,7 @@
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
@@ -28015,7 +28015,7 @@
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M339" t="inlineStr">
@@ -28097,7 +28097,7 @@
       </c>
       <c r="L340" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M340" t="inlineStr">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="L344" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M344" t="inlineStr">
@@ -28507,7 +28507,7 @@
       </c>
       <c r="L345" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M345" t="inlineStr">
@@ -28589,7 +28589,7 @@
       </c>
       <c r="L346" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M346" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="L347" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M347" t="inlineStr">
@@ -28753,7 +28753,7 @@
       </c>
       <c r="L348" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M348" t="inlineStr">
@@ -28835,7 +28835,7 @@
       </c>
       <c r="L349" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M349" t="inlineStr">
@@ -28917,7 +28917,7 @@
       </c>
       <c r="L350" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M350" t="inlineStr">
@@ -28999,7 +28999,7 @@
       </c>
       <c r="L351" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M351" t="inlineStr">
@@ -29081,7 +29081,7 @@
       </c>
       <c r="L352" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M352" t="inlineStr">
@@ -29143,7 +29143,7 @@
       </c>
       <c r="L353" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M353" t="inlineStr">
@@ -29391,7 +29391,7 @@
       </c>
       <c r="L357" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M357" t="inlineStr">
@@ -29639,7 +29639,7 @@
       </c>
       <c r="L361" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M361" t="inlineStr">
@@ -29743,7 +29743,7 @@
       </c>
       <c r="L363" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M363" t="inlineStr">
@@ -29795,7 +29795,7 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -29847,7 +29847,7 @@
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M365" t="inlineStr">
@@ -29899,7 +29899,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M366" t="inlineStr">
@@ -29951,7 +29951,7 @@
       </c>
       <c r="L367" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M367" t="inlineStr">
@@ -30003,7 +30003,7 @@
       </c>
       <c r="L368" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M368" t="inlineStr">
@@ -30060,7 +30060,7 @@
       </c>
       <c r="L369" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="M369" t="inlineStr">

</xml_diff>

<commit_message>
Edit a resistance rule
</commit_message>
<xml_diff>
--- a/cellstocks/data/admin.xlsx
+++ b/cellstocks/data/admin.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1846,7 +1846,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -3280,7 +3280,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -5196,7 +5196,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -6200,7 +6200,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -6692,7 +6692,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -6774,7 +6774,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -6856,7 +6856,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -6938,7 +6938,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -7686,7 +7686,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -7768,7 +7768,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -7850,7 +7850,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -7932,7 +7932,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -8096,7 +8096,7 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -8260,7 +8260,7 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -8506,7 +8506,7 @@
       </c>
       <c r="M102" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -8588,7 +8588,7 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="M106" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -8926,7 +8926,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -9008,7 +9008,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -9172,7 +9172,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -9254,7 +9254,7 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -9336,7 +9336,7 @@
       </c>
       <c r="M112" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -9500,7 +9500,7 @@
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="M116" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="M117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="M119" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -10156,7 +10156,7 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -10238,7 +10238,7 @@
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -10320,7 +10320,7 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -10566,7 +10566,7 @@
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -10648,7 +10648,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -10730,7 +10730,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -10812,7 +10812,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -10894,7 +10894,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
@@ -10976,7 +10976,7 @@
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N132" t="inlineStr">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N133" t="inlineStr">
@@ -11140,7 +11140,7 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N134" t="inlineStr">
@@ -11222,7 +11222,7 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="M145" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -12124,7 +12124,7 @@
       </c>
       <c r="M146" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -12206,7 +12206,7 @@
       </c>
       <c r="M147" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -12288,7 +12288,7 @@
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -12370,7 +12370,7 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -12452,7 +12452,7 @@
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -12534,7 +12534,7 @@
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -12616,7 +12616,7 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -12698,7 +12698,7 @@
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -12780,7 +12780,7 @@
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -12867,7 +12867,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
@@ -13123,7 +13123,7 @@
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
@@ -13369,7 +13369,7 @@
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N165" t="inlineStr">
@@ -14281,7 +14281,7 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N172" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="M174" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N174" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N175" t="inlineStr">
@@ -14609,7 +14609,7 @@
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
@@ -14691,7 +14691,7 @@
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
@@ -14855,7 +14855,7 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N179" t="inlineStr">
@@ -14937,7 +14937,7 @@
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N180" t="inlineStr">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
@@ -15101,7 +15101,7 @@
       </c>
       <c r="M182" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N182" t="inlineStr">
@@ -15193,7 +15193,7 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N185" t="inlineStr">
@@ -15449,7 +15449,7 @@
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
@@ -15541,7 +15541,7 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N188" t="inlineStr">
@@ -15715,7 +15715,7 @@
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N189" t="inlineStr">
@@ -17273,7 +17273,7 @@
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N208" t="inlineStr">
@@ -17355,7 +17355,7 @@
       </c>
       <c r="M209" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N209" t="inlineStr">
@@ -17437,7 +17437,7 @@
       </c>
       <c r="M210" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N210" t="inlineStr">
@@ -17519,7 +17519,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N211" t="inlineStr">
@@ -17601,7 +17601,7 @@
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
@@ -17693,7 +17693,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
@@ -17775,7 +17775,7 @@
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N214" t="inlineStr">
@@ -17857,7 +17857,7 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
@@ -17949,7 +17949,7 @@
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
@@ -18041,7 +18041,7 @@
       </c>
       <c r="M217" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N217" t="inlineStr">
@@ -18123,7 +18123,7 @@
       </c>
       <c r="M218" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N218" t="inlineStr">
@@ -18205,7 +18205,7 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N219" t="inlineStr">
@@ -18287,7 +18287,7 @@
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N220" t="inlineStr">
@@ -18369,7 +18369,7 @@
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N221" t="inlineStr">
@@ -18451,7 +18451,7 @@
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
@@ -18533,7 +18533,7 @@
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N223" t="inlineStr">
@@ -18615,7 +18615,7 @@
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N224" t="inlineStr">
@@ -18697,7 +18697,7 @@
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N225" t="inlineStr">
@@ -18779,7 +18779,7 @@
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N226" t="inlineStr">
@@ -18861,7 +18861,7 @@
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N227" t="inlineStr">
@@ -18943,7 +18943,7 @@
       </c>
       <c r="M228" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N228" t="inlineStr">
@@ -19025,7 +19025,7 @@
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N229" t="inlineStr">
@@ -19107,7 +19107,7 @@
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N230" t="inlineStr">
@@ -19189,7 +19189,7 @@
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N231" t="inlineStr">
@@ -19271,7 +19271,7 @@
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -19353,7 +19353,7 @@
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N233" t="inlineStr">
@@ -19435,7 +19435,7 @@
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N234" t="inlineStr">
@@ -19517,7 +19517,7 @@
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N235" t="inlineStr">
@@ -19599,7 +19599,7 @@
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N236" t="inlineStr">
@@ -19681,7 +19681,7 @@
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N237" t="inlineStr">
@@ -19763,7 +19763,7 @@
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N238" t="inlineStr">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="M239" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N239" t="inlineStr">
@@ -19927,7 +19927,7 @@
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N240" t="inlineStr">
@@ -20004,7 +20004,7 @@
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N241" t="inlineStr">
@@ -20081,7 +20081,7 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N242" t="inlineStr">
@@ -20163,7 +20163,7 @@
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N243" t="inlineStr">
@@ -20245,7 +20245,7 @@
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N244" t="inlineStr">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N245" t="inlineStr">
@@ -20409,7 +20409,7 @@
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N246" t="inlineStr">
@@ -20486,7 +20486,7 @@
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N247" t="inlineStr">
@@ -20568,7 +20568,7 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N248" t="inlineStr">
@@ -20650,7 +20650,7 @@
       </c>
       <c r="M249" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N249" t="inlineStr">
@@ -20732,7 +20732,7 @@
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N250" t="inlineStr">
@@ -20814,7 +20814,7 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N251" t="inlineStr">
@@ -20896,7 +20896,7 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N252" t="inlineStr">
@@ -20978,7 +20978,7 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N253" t="inlineStr">
@@ -21142,7 +21142,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N255" t="inlineStr">
@@ -21224,7 +21224,7 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N256" t="inlineStr">
@@ -21388,7 +21388,7 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N258" t="inlineStr">
@@ -21470,7 +21470,7 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N259" t="inlineStr">
@@ -21552,7 +21552,7 @@
       </c>
       <c r="M260" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N260" t="inlineStr">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="M261" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N261" t="inlineStr">
@@ -22203,7 +22203,7 @@
       </c>
       <c r="M268" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N268" t="inlineStr">
@@ -22280,7 +22280,7 @@
       </c>
       <c r="M269" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N269" t="inlineStr">
@@ -22362,7 +22362,7 @@
       </c>
       <c r="M270" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N270" t="inlineStr">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="M271" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N271" t="inlineStr">
@@ -23254,7 +23254,7 @@
       </c>
       <c r="M281" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N281" t="inlineStr">
@@ -23336,7 +23336,7 @@
       </c>
       <c r="M282" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N282" t="inlineStr">
@@ -23418,7 +23418,7 @@
       </c>
       <c r="M283" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N283" t="inlineStr">
@@ -23500,7 +23500,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N284" t="inlineStr">
@@ -23582,7 +23582,7 @@
       </c>
       <c r="M285" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N285" t="inlineStr">
@@ -23664,7 +23664,7 @@
       </c>
       <c r="M286" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N286" t="inlineStr">
@@ -23746,7 +23746,7 @@
       </c>
       <c r="M287" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N287" t="inlineStr">
@@ -23828,7 +23828,7 @@
       </c>
       <c r="M288" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N288" t="inlineStr">
@@ -23910,7 +23910,7 @@
       </c>
       <c r="M289" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N289" t="inlineStr">
@@ -23987,7 +23987,7 @@
       </c>
       <c r="M290" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N290" t="inlineStr">
@@ -24069,7 +24069,7 @@
       </c>
       <c r="M291" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N291" t="inlineStr">
@@ -24151,7 +24151,7 @@
       </c>
       <c r="M292" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N292" t="inlineStr">
@@ -24233,7 +24233,7 @@
       </c>
       <c r="M293" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N293" t="inlineStr">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="M294" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N294" t="inlineStr">
@@ -24397,7 +24397,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -24479,7 +24479,7 @@
       </c>
       <c r="M296" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N296" t="inlineStr">
@@ -24561,7 +24561,7 @@
       </c>
       <c r="M297" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N297" t="inlineStr">
@@ -24643,7 +24643,7 @@
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -24971,7 +24971,7 @@
       </c>
       <c r="M302" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N302" t="inlineStr">
@@ -25053,7 +25053,7 @@
       </c>
       <c r="M303" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N303" t="inlineStr">
@@ -25463,7 +25463,7 @@
       </c>
       <c r="M308" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N308" t="inlineStr">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="M309" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N309" t="inlineStr">
@@ -25627,7 +25627,7 @@
       </c>
       <c r="M310" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N310" t="inlineStr">
@@ -25709,7 +25709,7 @@
       </c>
       <c r="M311" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N311" t="inlineStr">
@@ -25791,7 +25791,7 @@
       </c>
       <c r="M312" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N312" t="inlineStr">
@@ -25873,7 +25873,7 @@
       </c>
       <c r="M313" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N313" t="inlineStr">
@@ -25955,7 +25955,7 @@
       </c>
       <c r="M314" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N314" t="inlineStr">
@@ -26037,7 +26037,7 @@
       </c>
       <c r="M315" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N315" t="inlineStr">
@@ -26119,7 +26119,7 @@
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
@@ -26201,7 +26201,7 @@
       </c>
       <c r="M317" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N317" t="inlineStr">
@@ -26283,7 +26283,7 @@
       </c>
       <c r="M318" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N318" t="inlineStr">
@@ -26365,7 +26365,7 @@
       </c>
       <c r="M319" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N319" t="inlineStr">
@@ -26447,7 +26447,7 @@
       </c>
       <c r="M320" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N320" t="inlineStr">
@@ -26529,7 +26529,7 @@
       </c>
       <c r="M321" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N321" t="inlineStr">
@@ -26611,7 +26611,7 @@
       </c>
       <c r="M322" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N322" t="inlineStr">
@@ -26693,7 +26693,7 @@
       </c>
       <c r="M323" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N323" t="inlineStr">
@@ -26775,7 +26775,7 @@
       </c>
       <c r="M324" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N324" t="inlineStr">
@@ -26857,7 +26857,7 @@
       </c>
       <c r="M325" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N325" t="inlineStr">
@@ -26939,7 +26939,7 @@
       </c>
       <c r="M326" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N326" t="inlineStr">
@@ -27031,7 +27031,7 @@
       </c>
       <c r="M327" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N327" t="inlineStr">
@@ -27123,7 +27123,7 @@
       </c>
       <c r="M328" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N328" t="inlineStr">
@@ -27205,7 +27205,7 @@
       </c>
       <c r="M329" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N329" t="inlineStr">
@@ -27287,7 +27287,7 @@
       </c>
       <c r="M330" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N330" t="inlineStr">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="M331" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N331" t="inlineStr">
@@ -27451,7 +27451,7 @@
       </c>
       <c r="M332" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N332" t="inlineStr">
@@ -27528,7 +27528,7 @@
       </c>
       <c r="M333" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N333" t="inlineStr">
@@ -27610,7 +27610,7 @@
       </c>
       <c r="M334" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N334" t="inlineStr">
@@ -27692,7 +27692,7 @@
       </c>
       <c r="M335" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N335" t="inlineStr">
@@ -27774,7 +27774,7 @@
       </c>
       <c r="M336" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N336" t="inlineStr">
@@ -27856,7 +27856,7 @@
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
@@ -27938,7 +27938,7 @@
       </c>
       <c r="M338" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N338" t="inlineStr">
@@ -28020,7 +28020,7 @@
       </c>
       <c r="M339" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N339" t="inlineStr">
@@ -28102,7 +28102,7 @@
       </c>
       <c r="M340" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N340" t="inlineStr">
@@ -28184,7 +28184,7 @@
       </c>
       <c r="M341" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N341" t="inlineStr">
@@ -28266,7 +28266,7 @@
       </c>
       <c r="M342" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N342" t="inlineStr">
@@ -28348,7 +28348,7 @@
       </c>
       <c r="M343" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N343" t="inlineStr">
@@ -28922,7 +28922,7 @@
       </c>
       <c r="M350" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N350" t="inlineStr">
@@ -29148,7 +29148,7 @@
       </c>
       <c r="M353" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N353" t="inlineStr">
@@ -29210,7 +29210,7 @@
       </c>
       <c r="M354" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N354" t="inlineStr">
@@ -29272,7 +29272,7 @@
       </c>
       <c r="M355" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N355" t="inlineStr">
@@ -29334,7 +29334,7 @@
       </c>
       <c r="M356" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N356" t="inlineStr">
@@ -29396,7 +29396,7 @@
       </c>
       <c r="M357" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N357" t="inlineStr">
@@ -29458,7 +29458,7 @@
       </c>
       <c r="M358" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N358" t="inlineStr">
@@ -29520,7 +29520,7 @@
       </c>
       <c r="M359" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N359" t="inlineStr">
@@ -29582,7 +29582,7 @@
       </c>
       <c r="M360" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N360" t="inlineStr">
@@ -29644,7 +29644,7 @@
       </c>
       <c r="M361" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N361" t="inlineStr">
@@ -29696,7 +29696,7 @@
       </c>
       <c r="M362" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N362" t="inlineStr">
@@ -29748,7 +29748,7 @@
       </c>
       <c r="M363" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N363" t="inlineStr">
@@ -29800,7 +29800,7 @@
       </c>
       <c r="M364" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N364" t="inlineStr">
@@ -29852,7 +29852,7 @@
       </c>
       <c r="M365" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N365" t="inlineStr">
@@ -29904,7 +29904,7 @@
       </c>
       <c r="M366" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N366" t="inlineStr">
@@ -29956,7 +29956,7 @@
       </c>
       <c r="M367" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N367" t="inlineStr">
@@ -30008,7 +30008,7 @@
       </c>
       <c r="M368" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N368" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="M369" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N369" t="inlineStr">

</xml_diff>